<commit_message>
feat: add new site automation
</commit_message>
<xml_diff>
--- a/templates/www.teseu.net_admin_template.xlsx
+++ b/templates/www.teseu.net_admin_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias/EliasLi/03.code-github/formfiller-excel-chrome/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998AF65D-11CA-334B-B761-46FC1CFB6E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DAFF1E3-E215-FD4B-A6A4-8ABD9C399B80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3540" yWindow="3880" windowWidth="24780" windowHeight="17180" xr2:uid="{90DC7538-4C1F-0E40-A7F3-11B48F1F7614}"/>
+    <workbookView xWindow="4280" yWindow="2460" windowWidth="24780" windowHeight="17180" xr2:uid="{90DC7538-4C1F-0E40-A7F3-11B48F1F7614}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -479,7 +479,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="B3">
         <v>2026</v>
@@ -499,7 +499,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="B4">
         <v>2026</v>
@@ -518,144 +518,25 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>655</v>
-      </c>
-      <c r="B5">
-        <v>2026</v>
-      </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="D5">
-        <v>20</v>
-      </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5">
-        <v>6</v>
-      </c>
+      <c r="A5" s="1"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>656</v>
-      </c>
-      <c r="B6">
-        <v>2026</v>
-      </c>
-      <c r="C6">
-        <v>3</v>
-      </c>
-      <c r="D6">
-        <v>21</v>
-      </c>
-      <c r="E6">
-        <v>7</v>
-      </c>
-      <c r="F6">
-        <v>7</v>
-      </c>
+      <c r="A6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>657</v>
-      </c>
-      <c r="B7">
-        <v>2026</v>
-      </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="D7">
-        <v>22</v>
-      </c>
-      <c r="E7">
-        <v>8</v>
-      </c>
-      <c r="F7">
-        <v>8</v>
-      </c>
+      <c r="A7" s="1"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>658</v>
-      </c>
-      <c r="B8">
-        <v>2026</v>
-      </c>
-      <c r="C8">
-        <v>3</v>
-      </c>
-      <c r="D8">
-        <v>23</v>
-      </c>
-      <c r="E8">
-        <v>9</v>
-      </c>
-      <c r="F8">
-        <v>9</v>
-      </c>
+      <c r="A8" s="1"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>659</v>
-      </c>
-      <c r="B9">
-        <v>2026</v>
-      </c>
-      <c r="C9">
-        <v>3</v>
-      </c>
-      <c r="D9">
-        <v>24</v>
-      </c>
-      <c r="E9">
-        <v>10</v>
-      </c>
-      <c r="F9">
-        <v>10</v>
-      </c>
+      <c r="A9" s="1"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>660</v>
-      </c>
-      <c r="B10">
-        <v>2026</v>
-      </c>
-      <c r="C10">
-        <v>3</v>
-      </c>
-      <c r="D10">
-        <v>25</v>
-      </c>
-      <c r="E10">
-        <v>11</v>
-      </c>
-      <c r="F10">
-        <v>11</v>
-      </c>
+      <c r="A10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>661</v>
-      </c>
-      <c r="B11">
-        <v>2026</v>
-      </c>
-      <c r="C11">
-        <v>3</v>
-      </c>
-      <c r="D11">
-        <v>26</v>
-      </c>
-      <c r="E11">
-        <v>12</v>
-      </c>
-      <c r="F11">
-        <v>12</v>
-      </c>
+      <c r="A11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>